<commit_message>
Require calibration parameter readback before success
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/EspLink/EspLink_Validation.xlsx
+++ b/Firmware/Modules/EspLink/EspLink_Validation.xlsx
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1583,6 +1583,89 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>EL-013</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>کالیبراسیون و read-back</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>بالا</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Firmware جدید + لینک فعال</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>از کارت کالیبراسیون ID0..6 را ارسال کن؛ هر مقدار باید بعد از تأیید قبلی فرستاده شود</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>ID0..6؛ مقدار متفاوت</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>حداکثر 20s</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 فقط صف است؛ موفقیت فقط پس از PARAM_REPORT/PARAMS_BULK با مقدار عیناً برابر</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>پس از ریست، NVM</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>هر 7 مقدار read-back برابر؛ پس از حدود 2s و reset مقادیر باقی بماند</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>Host PASS: test_panel_calibration_requires_readback_v127 + NVM ids 0..6؛ برد اجرا نشده</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>Host جای تست برد را نمی‌گیرد؛ برد باید با build جدید فلش شود</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>Firmware/Modules/Charger/Tester/host_test_charger.py؛ tools/check_firmware_syntax.sh</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>WORKTREE</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr"/>
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:Q3"/>
@@ -1590,10 +1673,10 @@
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="L5:L16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L5:L17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>='فهرست‌ها'!$A$2:$A$6</formula1>
     </dataValidation>
-    <dataValidation sqref="C5:C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C5:C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>='فهرست‌ها'!$B$9:$B$11</formula1>
     </dataValidation>
   </dataValidations>
@@ -2046,7 +2129,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
@@ -2109,7 +2192,7 @@
         </is>
       </c>
       <c r="B17" s="6">
-        <f>IF(12=0,0,COUNTIF('برنامه تست'!L:L,"قبول")/12)</f>
+        <f>IF(13=0,0,COUNTIF('برنامه تست'!L:L,"قبول")/13)</f>
         <v/>
       </c>
       <c r="C17" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Gate LUT pushes on calibration readback
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/EspLink/EspLink_Validation.xlsx
+++ b/Firmware/Modules/EspLink/EspLink_Validation.xlsx
@@ -16,7 +16,7 @@
     <sheet name="ماشین حالت" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -1689,7 +1689,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>از پنل قبل از ارسال /lut/read را بزن؛ سپس یک جدول هر دو باتری را push و commit کن؛ بعد از commit و reset دوباره /lut/read را بزن</t>
+          <t>از پنل «خواندن جدول فعلی» را بزن؛ سپس update هر دو باتری را با gain/offset متفاوت اجرا کن؛ بعد از commit و reset دوباره /lut/read و تله‌متری را بزن</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>STM32 برای هر دو کانال LUT_DATA واقعی می‌فرستد؛ پنل ستون فعلی، پیشنهادی و پس از commit را نشان می‌دهد؛ صفرنقطه برای حذف override معتبر است.</t>
+          <t>STM32 برای هر دو کانال LUT_DATA واقعی می‌فرستد؛ gain/offset هر چهار شناسه پیش از LUT با readback تأیید می‌شود؛ پنل ستون فعلی، پیشنهادی و پس از commit را نشان می‌دهد؛ صفرنقطه برای حذف override معتبر است.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 307 check؛ اجرای برد فیزیکی انجام نشده</t>
+          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 316 check؛ شامل preflight و readback gain/offset؛ اجرای برد فیزیکی انجام نشده</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>یک کانال معتبر و یک کانال بدون جدول/نامعتبر را pack کن؛ قبل و بعد از commit LUT_READ بگیر</t>
+          <t>یک update تکی برای باتری ۱ یا ۲ با یک کانال معتبر و یک کانال بدون جدول/نامعتبر اجرا کن؛ قبل و بعد از commit LUT_READ و readback gain/offset بگیر</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>count=0 معتبر است؛ حذف override به‌صورت changed-confirmed دیده می‌شود؛ نقطهٔ اضافه mismatch و readback خطادار failure است</t>
+          <t>count=0 معتبر است؛ حذف override به‌صورت changed-confirmed دیده می‌شود؛ نقطهٔ اضافه mismatch و readback خطادار failure است؛ خطای gain/offset قبل از POST /lut جلوی جدول را می‌گیرد.</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 307 check؛ اجرای برد فیزیکی انجام نشده</t>
+          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 316 check؛ شامل گیت readback و update مستقل؛ اجرای برد فیزیکی انجام نشده</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
@@ -1873,7 +1873,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2265,7 +2264,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
@@ -2371,7 +2369,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
@@ -2444,7 +2441,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
@@ -2473,7 +2469,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
@@ -2535,7 +2530,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Apply calibration as one confirmed readback batch
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/EspLink/EspLink_Validation.xlsx
+++ b/Firmware/Modules/EspLink/EspLink_Validation.xlsx
@@ -1606,7 +1606,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>از کارت کالیبراسیون ID0..6 را ارسال کن؛ هر مقدار باید بعد از تأیید قبلی فرستاده شود</t>
+          <t>از کارت کالیبراسیون یک batch شامل همهٔ پارامترهای معتبر (ID0..6) را با یک تأیید ارسال کن؛ هر مقدار باید پس از تأیید قبلی فرستاده شود</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1631,12 +1631,12 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>هر 7 مقدار read-back برابر؛ پس از حدود 2s و reset مقادیر باقی بماند</t>
+          <t>هر ۷ مقدار معتبر read-back برابر؛ وضعیت هر نام unchanged/changed-confirmed/mismatch/readback failure؛ پس از حدود ۲s و reset مقادیر باقی بماند</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: test_panel_calibration_requires_readback_v127 + NVM ids 0..6؛ برد اجرا نشده</t>
+          <t>Host PASS: DOM 316 check شامل summary نام‌محور، modal یک‌تأییدی و write/readback همهٔ پارامترهای معتبر؛ Charger 53 check؛ برد اجرا نشده</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>از پنل «خواندن جدول فعلی» را بزن؛ سپس update هر دو باتری را با gain/offset متفاوت اجرا کن؛ بعد از commit و reset دوباره /lut/read و تله‌متری را بزن</t>
+          <t>از پنل «خواندن جدول فعلی» را بزن؛ سپس update هر دو باتری را اجرا کن؛ پارامترهای معتبر کالیبراسیونِ تراکنش (gain/offset باتری هدف + آفست‌های ولتاژ) یک‌جا قبل از LUT اعمال و readback شوند؛ بعد از commit و reset دوباره /lut/read و تله‌متری را بزن</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>STM32 برای هر دو کانال LUT_DATA واقعی می‌فرستد؛ gain/offset هر چهار شناسه پیش از LUT با readback تأیید می‌شود؛ پنل ستون فعلی، پیشنهادی و پس از commit را نشان می‌دهد؛ صفرنقطه برای حذف override معتبر است.</t>
+          <t>STM32 برای هر دو کانال LUT_DATA واقعی می‌فرستد؛ همهٔ پارامترهای معتبر کالیبراسیونِ تراکنش پیش از LUT با readback تأیید می‌شوند؛ پنل ستون فعلی، پیشنهادی و پس از commit را نشان می‌دهد؛ صفرنقطه برای حذف override معتبر است.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 316 check؛ شامل preflight و readback gain/offset؛ اجرای برد فیزیکی انجام نشده</t>
+          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 316 check؛ شامل preflight، readback همهٔ calibrationهای معتبر، modal نام‌محور و update مستقل؛ اجرای برد فیزیکی انجام نشده</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 316 check؛ شامل گیت readback و update مستقل؛ اجرای برد فیزیکی انجام نشده</t>
+          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 316 check؛ شامل گیت readback کالیبراسیون، update مستقل و summary صفرنقطه؛ اجرای برد فیزیکی انجام نشده</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Polish calibration sample selection controls
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/EspLink/EspLink_Validation.xlsx
+++ b/Firmware/Modules/EspLink/EspLink_Validation.xlsx
@@ -1636,7 +1636,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: DOM 316 check شامل summary نام‌محور، modal یک‌تأییدی و write/readback همهٔ پارامترهای معتبر؛ Charger 53 check؛ برد اجرا نشده</t>
+          <t>Host PASS: DOM 319 check شامل summary نام‌محور، checkbox انتخاب همهٔ نمونه‌ها، modal یک‌تأییدی و write/readback همهٔ پارامترهای معتبر؛ Charger 53 check؛ برد اجرا نشده</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 316 check؛ شامل preflight، readback همهٔ calibrationهای معتبر، modal نام‌محور و update مستقل؛ اجرای برد فیزیکی انجام نشده</t>
+          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 319 check؛ شامل preflight، readback همهٔ calibrationهای معتبر، checkbox نمونه‌ها، modal نام‌محور و update مستقل؛ اجرای برد فیزیکی انجام نشده</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 316 check؛ شامل گیت readback کالیبراسیون، update مستقل و summary صفرنقطه؛ اجرای برد فیزیکی انجام نشده</t>
+          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 319 check؛ شامل گیت readback کالیبراسیون، update مستقل، checkbox انتخاب نمونه و summary صفرنقطه؛ اجرای برد فیزیکی انجام نشده</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Separate bench sweep and manual duty controls
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/EspLink/EspLink_Validation.xlsx
+++ b/Firmware/Modules/EspLink/EspLink_Validation.xlsx
@@ -1636,7 +1636,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: DOM 319 check شامل summary نام‌محور، checkbox انتخاب همهٔ نمونه‌ها، modal یک‌تأییدی و write/readback همهٔ پارامترهای معتبر؛ Charger 53 check؛ برد اجرا نشده</t>
+          <t>Host PASS: DOM 322 check شامل summary نام‌محور، checkbox انتخاب همهٔ نمونه‌ها، modal یک‌تأییدی و write/readback همهٔ پارامترهای معتبر؛ Charger 53 check؛ برد اجرا نشده</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 319 check؛ شامل preflight، readback همهٔ calibrationهای معتبر، checkbox نمونه‌ها، modal نام‌محور و update مستقل؛ اجرای برد فیزیکی انجام نشده</t>
+          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 322 check؛ شامل preflight، readback همهٔ calibrationهای معتبر، انتخاب انحصاری SWEEP/دستی با گام، modal نام‌محور و update مستقل؛ اجرای برد فیزیکی انجام نشده</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 319 check؛ شامل گیت readback کالیبراسیون، update مستقل، checkbox انتخاب نمونه و summary صفرنقطه؛ اجرای برد فیزیکی انجام نشده</t>
+          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 322 check؛ شامل گیت readback کالیبراسیون، update مستقل، checkbox انتخاب نمونه و summary صفرنقطه؛ اجرای برد فیزیکی انجام نشده</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Unify factory reset button layout across settings
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/EspLink/EspLink_Validation.xlsx
+++ b/Firmware/Modules/EspLink/EspLink_Validation.xlsx
@@ -1636,7 +1636,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: DOM 322 check شامل summary نام‌محور، checkbox انتخاب همهٔ نمونه‌ها، modal یک‌تأییدی و write/readback همهٔ پارامترهای معتبر؛ Charger 53 check؛ برد اجرا نشده</t>
+          <t>Host PASS: DOM 324 check شامل summary نام‌محور، checkbox انتخاب همهٔ نمونه‌ها، modal یک‌تأییدی و write/readback همهٔ پارامترهای معتبر؛ Charger 53 check؛ برد اجرا نشده</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 322 check؛ شامل preflight، readback همهٔ calibrationهای معتبر، انتخاب انحصاری SWEEP/دستی با گام، modal نام‌محور و update مستقل؛ اجرای برد فیزیکی انجام نشده</t>
+          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 324 check؛ شامل preflight، readback همهٔ calibrationهای معتبر، انتخاب انحصاری SWEEP/دستی با گام، تم کلیدهای پنل و update مستقل؛ اجرای برد فیزیکی انجام نشده</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 322 check؛ شامل گیت readback کالیبراسیون، update مستقل، checkbox انتخاب نمونه و summary صفرنقطه؛ اجرای برد فیزیکی انجام نشده</t>
+          <t>Host PASS: CalLut 159 check، ESP 112 check، DOM پنل 324 check؛ شامل گیت readback کالیبراسیون، update مستقل، کلیدهای factory-reset یکدست و summary صفرنقطه؛ اجرای برد فیزیکی انجام نشده</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">

</xml_diff>